<commit_message>
Excel de etiquetas: linha do meio mais grossa nas duas colunas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KBPpTkmjFG3PHLcKCudDC4
</commit_message>
<xml_diff>
--- a/etiquetas/etiquetas-A01-A84-B01-B168-70x40.xlsx
+++ b/etiquetas/etiquetas-A01-A84-B01-B168-70x40.xlsx
@@ -41,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -50,7 +50,14 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
+      <right style="medium">
+        <color rgb="00000000"/>
+      </right>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00000000"/>
+      </left>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -58,10 +65,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>

</xml_diff>